<commit_message>
Update Level 3 structure analysis results
- Fix Level 3 (Structure) CI indicators
- Recomputed for all 600 network instances
</commit_message>
<xml_diff>
--- a/outputs/results/level3_structure.xlsx
+++ b/outputs/results/level3_structure.xlsx
@@ -538,7 +538,7 @@
         <v>8089076.106618579</v>
       </c>
       <c r="D2" t="n">
-        <v>9369385.508193471</v>
+        <v>9369385.508193472</v>
       </c>
       <c r="E2" t="n">
         <v>13710583.37808686</v>
@@ -553,13 +553,13 @@
         <v>19932508.62290131</v>
       </c>
       <c r="I2" t="n">
-        <v>26293315.8589543</v>
+        <v>26293315.85895429</v>
       </c>
       <c r="J2" t="n">
         <v>25094655.72969376</v>
       </c>
       <c r="K2" t="n">
-        <v>24854503.38681489</v>
+        <v>24854503.38681488</v>
       </c>
       <c r="L2" t="n">
         <v>36917827.86010224</v>
@@ -574,7 +574,7 @@
         <v>42644107.58540097</v>
       </c>
       <c r="P2" t="n">
-        <v>40353782.7893723</v>
+        <v>40353782.78937231</v>
       </c>
       <c r="Q2" t="n">
         <v>44485518.81073952</v>
@@ -586,7 +586,7 @@
         <v>50735903.71122898</v>
       </c>
       <c r="T2" t="n">
-        <v>46017152.41885409</v>
+        <v>46017152.4188541</v>
       </c>
       <c r="U2" t="n">
         <v>50090167.04251139</v>
@@ -606,7 +606,7 @@
         <v>131347749.3133693</v>
       </c>
       <c r="D3" t="n">
-        <v>161420770.2677201</v>
+        <v>161420770.26772</v>
       </c>
       <c r="E3" t="n">
         <v>187393840.394321</v>
@@ -618,13 +618,13 @@
         <v>260953962.8170411</v>
       </c>
       <c r="H3" t="n">
-        <v>275980848.9247519</v>
+        <v>275980848.9247518</v>
       </c>
       <c r="I3" t="n">
         <v>396944850.8297944</v>
       </c>
       <c r="J3" t="n">
-        <v>375719682.4362761</v>
+        <v>375719682.436276</v>
       </c>
       <c r="K3" t="n">
         <v>358872992.0320138</v>
@@ -633,7 +633,7 @@
         <v>410273290.5243412</v>
       </c>
       <c r="M3" t="n">
-        <v>486264420.408472</v>
+        <v>486264420.4084719</v>
       </c>
       <c r="N3" t="n">
         <v>498529006.8457162</v>
@@ -645,16 +645,16 @@
         <v>611290765.0766717</v>
       </c>
       <c r="Q3" t="n">
-        <v>637863134.2133365</v>
+        <v>637863134.2133366</v>
       </c>
       <c r="R3" t="n">
         <v>769961874.4370582</v>
       </c>
       <c r="S3" t="n">
-        <v>949486554.2481431</v>
+        <v>949486554.248143</v>
       </c>
       <c r="T3" t="n">
-        <v>953708412.9294255</v>
+        <v>953708412.9294257</v>
       </c>
       <c r="U3" t="n">
         <v>1220813789.389164</v>
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>91180292.67058656</v>
+        <v>91180292.67058653</v>
       </c>
       <c r="D4" t="n">
         <v>93710731.43943182</v>
       </c>
       <c r="E4" t="n">
-        <v>127936429.7818655</v>
+        <v>127936429.7818656</v>
       </c>
       <c r="F4" t="n">
         <v>130562601.9411123</v>
@@ -704,19 +704,19 @@
         <v>270915683.0565785</v>
       </c>
       <c r="N4" t="n">
-        <v>261690590.3248459</v>
+        <v>261690590.324846</v>
       </c>
       <c r="O4" t="n">
         <v>264076448.2557718</v>
       </c>
       <c r="P4" t="n">
-        <v>259063011.7783152</v>
+        <v>259063011.7783151</v>
       </c>
       <c r="Q4" t="n">
         <v>220216702.2795961</v>
       </c>
       <c r="R4" t="n">
-        <v>271546709.0999898</v>
+        <v>271546709.0999897</v>
       </c>
       <c r="S4" t="n">
         <v>236731532.7764496</v>
@@ -725,7 +725,7 @@
         <v>310324549.1480372</v>
       </c>
       <c r="U4" t="n">
-        <v>326503144.6826567</v>
+        <v>326503144.6826566</v>
       </c>
       <c r="V4" t="n">
         <v>290188420.7182325</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>95609587.17377956</v>
+        <v>95609587.17377955</v>
       </c>
       <c r="D5" t="n">
         <v>105127460.215259</v>
@@ -779,7 +779,7 @@
         <v>203579545.2815051</v>
       </c>
       <c r="O5" t="n">
-        <v>235141620.8482908</v>
+        <v>235141620.8482909</v>
       </c>
       <c r="P5" t="n">
         <v>215388608.6263999</v>
@@ -800,7 +800,7 @@
         <v>310999857.0636779</v>
       </c>
       <c r="V5" t="n">
-        <v>315166308.9594516</v>
+        <v>315166308.9594517</v>
       </c>
     </row>
     <row r="6">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15052158.1630512</v>
+        <v>15052158.16305119</v>
       </c>
       <c r="D6" t="n">
         <v>17483879.26999453</v>
@@ -829,13 +829,13 @@
         <v>35785157.60756402</v>
       </c>
       <c r="I6" t="n">
-        <v>41741078.30081034</v>
+        <v>41741078.30081033</v>
       </c>
       <c r="J6" t="n">
         <v>49908127.63232215</v>
       </c>
       <c r="K6" t="n">
-        <v>65093472.75710715</v>
+        <v>65093472.75710714</v>
       </c>
       <c r="L6" t="n">
         <v>75983614.99616677</v>
@@ -844,10 +844,10 @@
         <v>88507486.40154165</v>
       </c>
       <c r="N6" t="n">
-        <v>94952116.0320957</v>
+        <v>94952116.03209572</v>
       </c>
       <c r="O6" t="n">
-        <v>117351484.3424691</v>
+        <v>117351484.3424692</v>
       </c>
       <c r="P6" t="n">
         <v>114673052.576736</v>
@@ -868,7 +868,7 @@
         <v>178221366.0379065</v>
       </c>
       <c r="V6" t="n">
-        <v>219412987.5923862</v>
+        <v>219412987.5923863</v>
       </c>
     </row>
     <row r="7">
@@ -903,13 +903,13 @@
         <v>249483326.7696108</v>
       </c>
       <c r="K7" t="n">
-        <v>265462952.3761149</v>
+        <v>265462952.3761148</v>
       </c>
       <c r="L7" t="n">
         <v>374678461.9314855</v>
       </c>
       <c r="M7" t="n">
-        <v>458455918.2888142</v>
+        <v>458455918.2888141</v>
       </c>
       <c r="N7" t="n">
         <v>695789145.2026008</v>
@@ -933,7 +933,7 @@
         <v>1355393033.159672</v>
       </c>
       <c r="U7" t="n">
-        <v>1592533113.292864</v>
+        <v>1592533113.292863</v>
       </c>
       <c r="V7" t="n">
         <v>1735116831.425889</v>
@@ -959,10 +959,10 @@
         <v>47426880.96418355</v>
       </c>
       <c r="G8" t="n">
-        <v>67906445.50660077</v>
+        <v>67906445.50660075</v>
       </c>
       <c r="H8" t="n">
-        <v>77660438.13984132</v>
+        <v>77660438.13984133</v>
       </c>
       <c r="I8" t="n">
         <v>146613382.1711184</v>
@@ -974,7 +974,7 @@
         <v>150725183.2802164</v>
       </c>
       <c r="L8" t="n">
-        <v>167821883.4556418</v>
+        <v>167821883.4556419</v>
       </c>
       <c r="M8" t="n">
         <v>195178202.3831118</v>
@@ -986,7 +986,7 @@
         <v>233436077.064579</v>
       </c>
       <c r="P8" t="n">
-        <v>199914538.1966064</v>
+        <v>199914538.1966063</v>
       </c>
       <c r="Q8" t="n">
         <v>257946954.5357895</v>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3174513.13140152</v>
+        <v>3174513.131401521</v>
       </c>
       <c r="D9" t="n">
         <v>4534492.956168546</v>
@@ -1027,7 +1027,7 @@
         <v>8454638.281394038</v>
       </c>
       <c r="G9" t="n">
-        <v>9943382.498950802</v>
+        <v>9943382.4989508</v>
       </c>
       <c r="H9" t="n">
         <v>14938935.85072067</v>
@@ -1039,7 +1039,7 @@
         <v>21021011.84735128</v>
       </c>
       <c r="K9" t="n">
-        <v>29723170.36608676</v>
+        <v>29723170.36608675</v>
       </c>
       <c r="L9" t="n">
         <v>36571761.06002803</v>
@@ -1048,10 +1048,10 @@
         <v>43894631.68701424</v>
       </c>
       <c r="N9" t="n">
-        <v>43519855.59326237</v>
+        <v>43519855.59326236</v>
       </c>
       <c r="O9" t="n">
-        <v>46485300.66811918</v>
+        <v>46485300.66811917</v>
       </c>
       <c r="P9" t="n">
         <v>63807056.82663034</v>
@@ -1072,7 +1072,7 @@
         <v>107326047.751088</v>
       </c>
       <c r="V9" t="n">
-        <v>117009994.4846696</v>
+        <v>117009994.4846697</v>
       </c>
     </row>
     <row r="10">
@@ -1093,7 +1093,7 @@
         <v>16040722.15346637</v>
       </c>
       <c r="E10" t="n">
-        <v>22980631.49600732</v>
+        <v>22980631.49600733</v>
       </c>
       <c r="F10" t="n">
         <v>40184769.78048138</v>
@@ -1105,13 +1105,13 @@
         <v>60063834.8593042</v>
       </c>
       <c r="I10" t="n">
-        <v>62211369.21209677</v>
+        <v>62211369.21209675</v>
       </c>
       <c r="J10" t="n">
-        <v>71287870.82173459</v>
+        <v>71287870.82173461</v>
       </c>
       <c r="K10" t="n">
-        <v>87353652.18823332</v>
+        <v>87353652.18823333</v>
       </c>
       <c r="L10" t="n">
         <v>95188522.58968198</v>
@@ -1129,13 +1129,13 @@
         <v>245689636.5322077</v>
       </c>
       <c r="Q10" t="n">
-        <v>243599635.6291193</v>
+        <v>243599635.6291192</v>
       </c>
       <c r="R10" t="n">
         <v>305013614.0964722</v>
       </c>
       <c r="S10" t="n">
-        <v>390496504.9895162</v>
+        <v>390496504.9895163</v>
       </c>
       <c r="T10" t="n">
         <v>232205311.7938215</v>
@@ -1155,13 +1155,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2734386.034847916</v>
+        <v>2734386.034847917</v>
       </c>
       <c r="D11" t="n">
         <v>3064791.808031337</v>
       </c>
       <c r="E11" t="n">
-        <v>4362468.944781385</v>
+        <v>4362468.944781384</v>
       </c>
       <c r="F11" t="n">
         <v>4749754.458329445</v>
@@ -1209,10 +1209,10 @@
         <v>42494232.93512341</v>
       </c>
       <c r="U11" t="n">
-        <v>40310228.98659901</v>
+        <v>40310228.986599</v>
       </c>
       <c r="V11" t="n">
-        <v>34408893.59511455</v>
+        <v>34408893.59511454</v>
       </c>
     </row>
     <row r="12">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>42837998.76038154</v>
+        <v>42837998.76038153</v>
       </c>
       <c r="D12" t="n">
         <v>51422061.75497194</v>
       </c>
       <c r="E12" t="n">
-        <v>67287101.33908358</v>
+        <v>67287101.33908357</v>
       </c>
       <c r="F12" t="n">
         <v>100486360.4315338</v>
@@ -1238,7 +1238,7 @@
         <v>118237955.4139958</v>
       </c>
       <c r="H12" t="n">
-        <v>191846939.8431664</v>
+        <v>191846939.8431665</v>
       </c>
       <c r="I12" t="n">
         <v>204634255.1867394</v>
@@ -1253,7 +1253,7 @@
         <v>338083463.7572277</v>
       </c>
       <c r="M12" t="n">
-        <v>446803447.0656346</v>
+        <v>446803447.0656345</v>
       </c>
       <c r="N12" t="n">
         <v>227511439.354766</v>
@@ -1262,13 +1262,13 @@
         <v>257291926.302587</v>
       </c>
       <c r="P12" t="n">
-        <v>231221514.3304556</v>
+        <v>231221514.3304555</v>
       </c>
       <c r="Q12" t="n">
         <v>267906334.1321024</v>
       </c>
       <c r="R12" t="n">
-        <v>343032257.9017611</v>
+        <v>343032257.901761</v>
       </c>
       <c r="S12" t="n">
         <v>383601562.9194907</v>
@@ -1280,7 +1280,7 @@
         <v>441551732.2377663</v>
       </c>
       <c r="V12" t="n">
-        <v>492048678.0426318</v>
+        <v>492048678.0426317</v>
       </c>
     </row>
     <row r="13">
@@ -1312,13 +1312,13 @@
         <v>62286423.00383772</v>
       </c>
       <c r="J13" t="n">
-        <v>67610272.00739238</v>
+        <v>67610272.00739236</v>
       </c>
       <c r="K13" t="n">
-        <v>76208886.56410924</v>
+        <v>76208886.56410922</v>
       </c>
       <c r="L13" t="n">
-        <v>86712284.81298482</v>
+        <v>86712284.81298484</v>
       </c>
       <c r="M13" t="n">
         <v>89109054.99824175</v>
@@ -1359,7 +1359,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8781944.136452299</v>
+        <v>8781944.136452297</v>
       </c>
       <c r="D14" t="n">
         <v>7689950.941156195</v>
@@ -1380,13 +1380,13 @@
         <v>69215855.5509553</v>
       </c>
       <c r="J14" t="n">
-        <v>72880970.46986143</v>
+        <v>72880970.46986145</v>
       </c>
       <c r="K14" t="n">
         <v>92352115.65950462</v>
       </c>
       <c r="L14" t="n">
-        <v>94313594.73820151</v>
+        <v>94313594.7382015</v>
       </c>
       <c r="M14" t="n">
         <v>131390517.5568016</v>
@@ -1410,7 +1410,7 @@
         <v>78563774.98243906</v>
       </c>
       <c r="T14" t="n">
-        <v>75822095.341224</v>
+        <v>75822095.34122398</v>
       </c>
       <c r="U14" t="n">
         <v>87328493.28748396</v>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5121330.235214586</v>
+        <v>5121330.235214587</v>
       </c>
       <c r="D15" t="n">
         <v>5791002.318204209</v>
@@ -1448,7 +1448,7 @@
         <v>14681310.23266052</v>
       </c>
       <c r="J15" t="n">
-        <v>21999075.25871412</v>
+        <v>21999075.25871413</v>
       </c>
       <c r="K15" t="n">
         <v>25622488.3143478</v>
@@ -1466,7 +1466,7 @@
         <v>36264901.31261487</v>
       </c>
       <c r="P15" t="n">
-        <v>43127000.92504329</v>
+        <v>43127000.9250433</v>
       </c>
       <c r="Q15" t="n">
         <v>41633402.59942147</v>
@@ -1505,7 +1505,7 @@
         <v>33881861.31142543</v>
       </c>
       <c r="E16" t="n">
-        <v>52651936.04780458</v>
+        <v>52651936.04780457</v>
       </c>
       <c r="F16" t="n">
         <v>120154046.0570434</v>
@@ -1532,7 +1532,7 @@
         <v>2458942231.366152</v>
       </c>
       <c r="N16" t="n">
-        <v>2743950644.017837</v>
+        <v>2743950644.017838</v>
       </c>
       <c r="O16" t="n">
         <v>2597215294.374425</v>
@@ -1541,22 +1541,22 @@
         <v>2647765148.35173</v>
       </c>
       <c r="Q16" t="n">
-        <v>2214633205.970904</v>
+        <v>2214633205.970903</v>
       </c>
       <c r="R16" t="n">
-        <v>2032712949.211089</v>
+        <v>2032712949.211088</v>
       </c>
       <c r="S16" t="n">
-        <v>2403775322.611176</v>
+        <v>2403775322.611177</v>
       </c>
       <c r="T16" t="n">
         <v>3038007828.743534</v>
       </c>
       <c r="U16" t="n">
-        <v>3508956256.648134</v>
+        <v>3508956256.648133</v>
       </c>
       <c r="V16" t="n">
-        <v>3057748804.464915</v>
+        <v>3057748804.464916</v>
       </c>
     </row>
     <row r="17">
@@ -1606,19 +1606,19 @@
         <v>25811464.89563097</v>
       </c>
       <c r="P17" t="n">
-        <v>25897938.94020607</v>
+        <v>25897938.94020606</v>
       </c>
       <c r="Q17" t="n">
         <v>72634869.71613385</v>
       </c>
       <c r="R17" t="n">
-        <v>51486958.06044179</v>
+        <v>51486958.0604418</v>
       </c>
       <c r="S17" t="n">
         <v>49784313.44569885</v>
       </c>
       <c r="T17" t="n">
-        <v>53483267.7805118</v>
+        <v>53483267.78051181</v>
       </c>
       <c r="U17" t="n">
         <v>54463203.70570423</v>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18276511.24036584</v>
+        <v>18276511.24036583</v>
       </c>
       <c r="D18" t="n">
         <v>23230778.62046279</v>
@@ -1650,7 +1650,7 @@
         <v>66864361.25542285</v>
       </c>
       <c r="H18" t="n">
-        <v>83508294.88045919</v>
+        <v>83508294.88045917</v>
       </c>
       <c r="I18" t="n">
         <v>93180818.03655756</v>
@@ -1659,7 +1659,7 @@
         <v>102522866.2458831</v>
       </c>
       <c r="K18" t="n">
-        <v>122554060.3461398</v>
+        <v>122554060.3461399</v>
       </c>
       <c r="L18" t="n">
         <v>190981909.1365732</v>
@@ -1677,7 +1677,7 @@
         <v>256719316.8687094</v>
       </c>
       <c r="Q18" t="n">
-        <v>262361544.9090802</v>
+        <v>262361544.9090803</v>
       </c>
       <c r="R18" t="n">
         <v>289921130.0033575</v>
@@ -1706,13 +1706,13 @@
         <v>119079298.2707011</v>
       </c>
       <c r="D19" t="n">
-        <v>151781578.4075402</v>
+        <v>151781578.4075401</v>
       </c>
       <c r="E19" t="n">
         <v>194039289.5433621</v>
       </c>
       <c r="F19" t="n">
-        <v>287799704.4243935</v>
+        <v>287799704.4243936</v>
       </c>
       <c r="G19" t="n">
         <v>391197607.6963027</v>
@@ -1721,7 +1721,7 @@
         <v>482840974.146363</v>
       </c>
       <c r="I19" t="n">
-        <v>657503293.0558969</v>
+        <v>657503293.055897</v>
       </c>
       <c r="J19" t="n">
         <v>564091830.5903852</v>
@@ -1730,7 +1730,7 @@
         <v>614030331.9361007</v>
       </c>
       <c r="L19" t="n">
-        <v>931768419.7140894</v>
+        <v>931768419.7140895</v>
       </c>
       <c r="M19" t="n">
         <v>977402101.0301433</v>
@@ -1771,16 +1771,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>296062437.0352493</v>
+        <v>296062437.0352492</v>
       </c>
       <c r="D20" t="n">
         <v>445876976.1714553</v>
       </c>
       <c r="E20" t="n">
-        <v>575195311.283718</v>
+        <v>575195311.2837179</v>
       </c>
       <c r="F20" t="n">
-        <v>752452117.0284026</v>
+        <v>752452117.0284027</v>
       </c>
       <c r="G20" t="n">
         <v>1074662466.359285</v>
@@ -1798,13 +1798,13 @@
         <v>1613505615.247138</v>
       </c>
       <c r="L20" t="n">
-        <v>1975970824.875014</v>
+        <v>1975970824.875015</v>
       </c>
       <c r="M20" t="n">
         <v>2363331716.837193</v>
       </c>
       <c r="N20" t="n">
-        <v>2535960270.115351</v>
+        <v>2535960270.11535</v>
       </c>
       <c r="O20" t="n">
         <v>3529763238.796884</v>
@@ -1813,7 +1813,7 @@
         <v>3827036912.911461</v>
       </c>
       <c r="Q20" t="n">
-        <v>3623347714.503384</v>
+        <v>3623347714.503385</v>
       </c>
       <c r="R20" t="n">
         <v>3076740109.618378</v>
@@ -1839,10 +1839,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>49023684.80082682</v>
+        <v>49023684.80082683</v>
       </c>
       <c r="D21" t="n">
-        <v>61795192.2257522</v>
+        <v>61795192.22575219</v>
       </c>
       <c r="E21" t="n">
         <v>80488102.43893544</v>
@@ -1857,22 +1857,22 @@
         <v>247046016.5014276</v>
       </c>
       <c r="I21" t="n">
-        <v>304226584.5912466</v>
+        <v>304226584.5912467</v>
       </c>
       <c r="J21" t="n">
         <v>312123435.7805789</v>
       </c>
       <c r="K21" t="n">
-        <v>381978838.2133775</v>
+        <v>381978838.2133774</v>
       </c>
       <c r="L21" t="n">
-        <v>396776830.9062691</v>
+        <v>396776830.906269</v>
       </c>
       <c r="M21" t="n">
         <v>550695431.22047</v>
       </c>
       <c r="N21" t="n">
-        <v>873985752.2367756</v>
+        <v>873985752.2367759</v>
       </c>
       <c r="O21" t="n">
         <v>435917093.934881</v>
@@ -1881,13 +1881,13 @@
         <v>383347498.0517201</v>
       </c>
       <c r="Q21" t="n">
-        <v>516464000.4185873</v>
+        <v>516464000.4185872</v>
       </c>
       <c r="R21" t="n">
         <v>625878652.6836627</v>
       </c>
       <c r="S21" t="n">
-        <v>629396499.8767853</v>
+        <v>629396499.8767854</v>
       </c>
       <c r="T21" t="n">
         <v>754322091.6598607</v>
@@ -1926,7 +1926,7 @@
         <v>15097638.15525361</v>
       </c>
       <c r="H22" t="n">
-        <v>19126905.66475866</v>
+        <v>19126905.66475865</v>
       </c>
       <c r="I22" t="n">
         <v>30458328.9380189</v>
@@ -1947,7 +1947,7 @@
         <v>69163912.72056906</v>
       </c>
       <c r="O22" t="n">
-        <v>74984265.36941108</v>
+        <v>74984265.36941107</v>
       </c>
       <c r="P22" t="n">
         <v>62233265.88095729</v>
@@ -1956,7 +1956,7 @@
         <v>80589757.20832242</v>
       </c>
       <c r="R22" t="n">
-        <v>75992276.42275424</v>
+        <v>75992276.42275423</v>
       </c>
       <c r="S22" t="n">
         <v>92168938.47970746</v>
@@ -1965,7 +1965,7 @@
         <v>111688794.5180051</v>
       </c>
       <c r="U22" t="n">
-        <v>125190141.5945238</v>
+        <v>125190141.5945237</v>
       </c>
       <c r="V22" t="n">
         <v>119424494.6066395</v>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>83339695.89055844</v>
+        <v>83339695.89055847</v>
       </c>
       <c r="D23" t="n">
         <v>94047092.09729242</v>
@@ -1991,7 +1991,7 @@
         <v>161663037.6740073</v>
       </c>
       <c r="G23" t="n">
-        <v>145784347.8946326</v>
+        <v>145784347.8946327</v>
       </c>
       <c r="H23" t="n">
         <v>204879662.2248192</v>
@@ -2062,7 +2062,7 @@
         <v>8714859.953926932</v>
       </c>
       <c r="H24" t="n">
-        <v>11352542.71200573</v>
+        <v>11352542.71200574</v>
       </c>
       <c r="I24" t="n">
         <v>17822271.23549733</v>
@@ -2074,10 +2074,10 @@
         <v>19271422.38463528</v>
       </c>
       <c r="L24" t="n">
-        <v>29629729.10194423</v>
+        <v>29629729.10194422</v>
       </c>
       <c r="M24" t="n">
-        <v>53781841.7634588</v>
+        <v>53781841.76345879</v>
       </c>
       <c r="N24" t="n">
         <v>65783974.68989968</v>
@@ -2086,13 +2086,13 @@
         <v>48671776.7875542</v>
       </c>
       <c r="P24" t="n">
-        <v>42472582.64989987</v>
+        <v>42472582.64989988</v>
       </c>
       <c r="Q24" t="n">
         <v>69116688.36001208</v>
       </c>
       <c r="R24" t="n">
-        <v>48693316.18326233</v>
+        <v>48693316.18326232</v>
       </c>
       <c r="S24" t="n">
         <v>56599984.13677145</v>
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>58702.70441102132</v>
+        <v>58702.70441102131</v>
       </c>
       <c r="D25" t="n">
         <v>162.6453287547363</v>
@@ -2130,10 +2130,10 @@
         <v>2066595.796239682</v>
       </c>
       <c r="H25" t="n">
-        <v>922068.875888811</v>
+        <v>922068.8758888112</v>
       </c>
       <c r="I25" t="n">
-        <v>3388662.33765169</v>
+        <v>3388662.337651689</v>
       </c>
       <c r="J25" t="n">
         <v>1855905.876194367</v>
@@ -2145,7 +2145,7 @@
         <v>4920244.93942196</v>
       </c>
       <c r="M25" t="n">
-        <v>5488027.718512474</v>
+        <v>5488027.718512473</v>
       </c>
       <c r="N25" t="n">
         <v>5936002.333532633</v>
@@ -2157,13 +2157,13 @@
         <v>5454195.469869311</v>
       </c>
       <c r="Q25" t="n">
-        <v>8206809.532071099</v>
+        <v>8206809.532071098</v>
       </c>
       <c r="R25" t="n">
         <v>9196135.673374588</v>
       </c>
       <c r="S25" t="n">
-        <v>7284906.347177562</v>
+        <v>7284906.347177561</v>
       </c>
       <c r="T25" t="n">
         <v>11213164.8909992</v>
@@ -2204,7 +2204,7 @@
         <v>30678256.82666358</v>
       </c>
       <c r="J26" t="n">
-        <v>29635889.23420216</v>
+        <v>29635889.23420215</v>
       </c>
       <c r="K26" t="n">
         <v>45384270.19336809</v>
@@ -2216,7 +2216,7 @@
         <v>57088613.80184861</v>
       </c>
       <c r="N26" t="n">
-        <v>83962354.81785229</v>
+        <v>83962354.81785227</v>
       </c>
       <c r="O26" t="n">
         <v>96897227.09566848</v>
@@ -2237,7 +2237,7 @@
         <v>84199098.04406445</v>
       </c>
       <c r="U26" t="n">
-        <v>77248218.10136767</v>
+        <v>77248218.10136765</v>
       </c>
       <c r="V26" t="n">
         <v>70736949.8649946</v>
@@ -2270,7 +2270,7 @@
         <v>5442658.832966417</v>
       </c>
       <c r="H27" t="n">
-        <v>6331167.932207854</v>
+        <v>6331167.932207852</v>
       </c>
       <c r="I27" t="n">
         <v>10124425.4790551</v>
@@ -2282,13 +2282,13 @@
         <v>26078182.83917569</v>
       </c>
       <c r="L27" t="n">
-        <v>33905726.93054552</v>
+        <v>33905726.93054551</v>
       </c>
       <c r="M27" t="n">
-        <v>44525777.48163019</v>
+        <v>44525777.48163018</v>
       </c>
       <c r="N27" t="n">
-        <v>46738853.29019572</v>
+        <v>46738853.29019571</v>
       </c>
       <c r="O27" t="n">
         <v>53993269.55030305</v>
@@ -2297,7 +2297,7 @@
         <v>48921815.56849898</v>
       </c>
       <c r="Q27" t="n">
-        <v>54398157.07649117</v>
+        <v>54398157.07649118</v>
       </c>
       <c r="R27" t="n">
         <v>52216055.58165036</v>
@@ -2312,7 +2312,7 @@
         <v>86469337.72897556</v>
       </c>
       <c r="V27" t="n">
-        <v>99523189.78109646</v>
+        <v>99523189.78109644</v>
       </c>
     </row>
     <row r="28">
@@ -2338,13 +2338,13 @@
         <v>38187058.95921374</v>
       </c>
       <c r="H28" t="n">
-        <v>58249817.30438238</v>
+        <v>58249817.30438236</v>
       </c>
       <c r="I28" t="n">
-        <v>76271953.81245892</v>
+        <v>76271953.8124589</v>
       </c>
       <c r="J28" t="n">
-        <v>110752095.9125498</v>
+        <v>110752095.9125497</v>
       </c>
       <c r="K28" t="n">
         <v>131895666.0449654</v>
@@ -2371,10 +2371,10 @@
         <v>463445635.2303671</v>
       </c>
       <c r="S28" t="n">
-        <v>539254149.5080038</v>
+        <v>539254149.5080037</v>
       </c>
       <c r="T28" t="n">
-        <v>624150398.5646961</v>
+        <v>624150398.5646962</v>
       </c>
       <c r="U28" t="n">
         <v>719296012.327747</v>
@@ -2391,10 +2391,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6528568.120521745</v>
+        <v>6528568.120521744</v>
       </c>
       <c r="D29" t="n">
-        <v>9835973.729831712</v>
+        <v>9835973.729831714</v>
       </c>
       <c r="E29" t="n">
         <v>12918083.55869793</v>
@@ -2424,7 +2424,7 @@
         <v>58536877.40379878</v>
       </c>
       <c r="N29" t="n">
-        <v>67777468.28006329</v>
+        <v>67777468.2800633</v>
       </c>
       <c r="O29" t="n">
         <v>136879133.7547396</v>
@@ -2439,13 +2439,13 @@
         <v>45740479.89380763</v>
       </c>
       <c r="S29" t="n">
-        <v>55647189.13855255</v>
+        <v>55647189.13855256</v>
       </c>
       <c r="T29" t="n">
         <v>54053075.44204865</v>
       </c>
       <c r="U29" t="n">
-        <v>58565706.64371127</v>
+        <v>58565706.64371126</v>
       </c>
       <c r="V29" t="n">
         <v>68977335.46919131</v>
@@ -2462,10 +2462,10 @@
         <v>17287611.5364555</v>
       </c>
       <c r="D30" t="n">
-        <v>25905772.4599278</v>
+        <v>25905772.45992779</v>
       </c>
       <c r="E30" t="n">
-        <v>53572689.51798952</v>
+        <v>53572689.51798953</v>
       </c>
       <c r="F30" t="n">
         <v>68303971.2569723</v>
@@ -2492,7 +2492,7 @@
         <v>740221741.5789728</v>
       </c>
       <c r="N30" t="n">
-        <v>1005723451.490698</v>
+        <v>1005723451.490697</v>
       </c>
       <c r="O30" t="n">
         <v>1285761888.522202</v>
@@ -2501,7 +2501,7 @@
         <v>1379391231.997006</v>
       </c>
       <c r="Q30" t="n">
-        <v>1456348202.451794</v>
+        <v>1456348202.451793</v>
       </c>
       <c r="R30" t="n">
         <v>1448801581.549375</v>
@@ -2533,10 +2533,10 @@
         <v>509021.4188416151</v>
       </c>
       <c r="E31" t="n">
-        <v>642276.7261651154</v>
+        <v>642276.7261651155</v>
       </c>
       <c r="F31" t="n">
-        <v>700949.1916011252</v>
+        <v>700949.1916011251</v>
       </c>
       <c r="G31" t="n">
         <v>872602.585445764</v>
@@ -2548,10 +2548,10 @@
         <v>2102676.475504752</v>
       </c>
       <c r="J31" t="n">
-        <v>3477948.924528629</v>
+        <v>3477948.924528628</v>
       </c>
       <c r="K31" t="n">
-        <v>3873257.768464414</v>
+        <v>3873257.768464413</v>
       </c>
       <c r="L31" t="n">
         <v>7462783.727399377</v>
@@ -2569,7 +2569,7 @@
         <v>10872593.85144398</v>
       </c>
       <c r="Q31" t="n">
-        <v>4683350.174821327</v>
+        <v>4683350.174821326</v>
       </c>
       <c r="R31" t="n">
         <v>5891234.881986796</v>
@@ -2581,7 +2581,7 @@
         <v>6745969.981314057</v>
       </c>
       <c r="U31" t="n">
-        <v>5968076.029595872</v>
+        <v>5968076.029595873</v>
       </c>
       <c r="V31" t="n">
         <v>6244236.442016692</v>
@@ -2696,7 +2696,7 @@
         <v>7488584.115713064</v>
       </c>
       <c r="D2" t="n">
-        <v>7794134.765424677</v>
+        <v>7794134.765424678</v>
       </c>
       <c r="E2" t="n">
         <v>10692066.71109403</v>
@@ -2711,7 +2711,7 @@
         <v>35318075.28935587</v>
       </c>
       <c r="I2" t="n">
-        <v>33988973.82412881</v>
+        <v>33988973.82412883</v>
       </c>
       <c r="J2" t="n">
         <v>35895793.18922643</v>
@@ -2729,7 +2729,7 @@
         <v>53067811.56004056</v>
       </c>
       <c r="O2" t="n">
-        <v>44434530.78223995</v>
+        <v>44434530.78223996</v>
       </c>
       <c r="P2" t="n">
         <v>47228794.16606884</v>
@@ -2764,7 +2764,7 @@
         <v>116203096.6876958</v>
       </c>
       <c r="D3" t="n">
-        <v>138817104.8722815</v>
+        <v>138817104.8722814</v>
       </c>
       <c r="E3" t="n">
         <v>165585349.2162463</v>
@@ -2785,7 +2785,7 @@
         <v>406169458.3036471</v>
       </c>
       <c r="K3" t="n">
-        <v>410432460.3958374</v>
+        <v>410432460.3958375</v>
       </c>
       <c r="L3" t="n">
         <v>413814128.466185</v>
@@ -2797,7 +2797,7 @@
         <v>490443728.0395266</v>
       </c>
       <c r="O3" t="n">
-        <v>482806630.5081751</v>
+        <v>482806630.5081753</v>
       </c>
       <c r="P3" t="n">
         <v>493891241.4578489</v>
@@ -2853,7 +2853,7 @@
         <v>138094632.4163843</v>
       </c>
       <c r="K4" t="n">
-        <v>142929007.9315824</v>
+        <v>142929007.9315823</v>
       </c>
       <c r="L4" t="n">
         <v>147443717.9324431</v>
@@ -2910,7 +2910,7 @@
         <v>47141040.63850641</v>
       </c>
       <c r="F5" t="n">
-        <v>59581161.46583804</v>
+        <v>59581161.46583803</v>
       </c>
       <c r="G5" t="n">
         <v>69164516.36273946</v>
@@ -2937,7 +2937,7 @@
         <v>83526199.67338553</v>
       </c>
       <c r="O5" t="n">
-        <v>99763453.51512824</v>
+        <v>99763453.51512823</v>
       </c>
       <c r="P5" t="n">
         <v>81833096.00353263</v>
@@ -2949,13 +2949,13 @@
         <v>122272668.9279727</v>
       </c>
       <c r="S5" t="n">
-        <v>121628216.8851765</v>
+        <v>121628216.8851766</v>
       </c>
       <c r="T5" t="n">
-        <v>98897256.27062716</v>
+        <v>98897256.27062717</v>
       </c>
       <c r="U5" t="n">
-        <v>105830596.6117924</v>
+        <v>105830596.6117923</v>
       </c>
       <c r="V5" t="n">
         <v>105550465.1622713</v>
@@ -2987,13 +2987,13 @@
         <v>47833395.24614199</v>
       </c>
       <c r="I6" t="n">
-        <v>50571349.35786528</v>
+        <v>50571349.35786526</v>
       </c>
       <c r="J6" t="n">
-        <v>59612053.4438791</v>
+        <v>59612053.44387908</v>
       </c>
       <c r="K6" t="n">
-        <v>77195272.39921437</v>
+        <v>77195272.39921436</v>
       </c>
       <c r="L6" t="n">
         <v>88461000.44713156</v>
@@ -3011,7 +3011,7 @@
         <v>142944925.1463386</v>
       </c>
       <c r="Q6" t="n">
-        <v>146393332.7245872</v>
+        <v>146393332.7245873</v>
       </c>
       <c r="R6" t="n">
         <v>167754330.2313487</v>
@@ -3023,7 +3023,7 @@
         <v>200782655.5048328</v>
       </c>
       <c r="U6" t="n">
-        <v>194906554.9711465</v>
+        <v>194906554.9711466</v>
       </c>
       <c r="V6" t="n">
         <v>175638737.3096682</v>
@@ -3037,22 +3037,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>41087666.02161234</v>
+        <v>41087666.02161235</v>
       </c>
       <c r="D7" t="n">
         <v>49487897.66252372</v>
       </c>
       <c r="E7" t="n">
-        <v>61499082.03081193</v>
+        <v>61499082.03081194</v>
       </c>
       <c r="F7" t="n">
-        <v>88335490.56300735</v>
+        <v>88335490.56300734</v>
       </c>
       <c r="G7" t="n">
         <v>144916718.9592466</v>
       </c>
       <c r="H7" t="n">
-        <v>233376591.7085166</v>
+        <v>233376591.7085165</v>
       </c>
       <c r="I7" t="n">
         <v>274627207.4832366</v>
@@ -3079,22 +3079,22 @@
         <v>625520308.5393764</v>
       </c>
       <c r="Q7" t="n">
-        <v>754258242.364375</v>
+        <v>754258242.3643751</v>
       </c>
       <c r="R7" t="n">
         <v>892043202.1441802</v>
       </c>
       <c r="S7" t="n">
-        <v>966081598.6447486</v>
+        <v>966081598.6447483</v>
       </c>
       <c r="T7" t="n">
-        <v>879213913.173574</v>
+        <v>879213913.1735737</v>
       </c>
       <c r="U7" t="n">
         <v>1006549220.109662</v>
       </c>
       <c r="V7" t="n">
-        <v>892622770.3737156</v>
+        <v>892622770.3737159</v>
       </c>
     </row>
     <row r="8">
@@ -3114,7 +3114,7 @@
         <v>31541420.51696195</v>
       </c>
       <c r="F8" t="n">
-        <v>45927682.76930612</v>
+        <v>45927682.76930611</v>
       </c>
       <c r="G8" t="n">
         <v>65687247.89968581</v>
@@ -3126,7 +3126,7 @@
         <v>138594886.3569572</v>
       </c>
       <c r="J8" t="n">
-        <v>146414792.2991922</v>
+        <v>146414792.2991923</v>
       </c>
       <c r="K8" t="n">
         <v>155458239.3098567</v>
@@ -3153,7 +3153,7 @@
         <v>238426829.2259613</v>
       </c>
       <c r="S8" t="n">
-        <v>314815809.6393555</v>
+        <v>314815809.6393556</v>
       </c>
       <c r="T8" t="n">
         <v>317838549.9331033</v>
@@ -3197,7 +3197,7 @@
         <v>17337744.87152448</v>
       </c>
       <c r="K9" t="n">
-        <v>23679504.5159116</v>
+        <v>23679504.51591161</v>
       </c>
       <c r="L9" t="n">
         <v>27738981.02252418</v>
@@ -3215,13 +3215,13 @@
         <v>53891976.35738254</v>
       </c>
       <c r="Q9" t="n">
-        <v>53280076.10492966</v>
+        <v>53280076.10492964</v>
       </c>
       <c r="R9" t="n">
         <v>48048776.77386909</v>
       </c>
       <c r="S9" t="n">
-        <v>69037450.82062307</v>
+        <v>69037450.82062308</v>
       </c>
       <c r="T9" t="n">
         <v>78413015.35366817</v>
@@ -3230,7 +3230,7 @@
         <v>99303684.93391035</v>
       </c>
       <c r="V9" t="n">
-        <v>92894259.64036542</v>
+        <v>92894259.64036541</v>
       </c>
     </row>
     <row r="10">
@@ -3266,13 +3266,13 @@
         <v>72187764.74941052</v>
       </c>
       <c r="J10" t="n">
-        <v>67205908.61885424</v>
+        <v>67205908.61885422</v>
       </c>
       <c r="K10" t="n">
         <v>102695611.8605617</v>
       </c>
       <c r="L10" t="n">
-        <v>74053075.4666606</v>
+        <v>74053075.46666059</v>
       </c>
       <c r="M10" t="n">
         <v>84083675.64672071</v>
@@ -3296,7 +3296,7 @@
         <v>442140396.247372</v>
       </c>
       <c r="T10" t="n">
-        <v>88367348.44745564</v>
+        <v>88367348.44745563</v>
       </c>
       <c r="U10" t="n">
         <v>102726785.3392245</v>
@@ -3316,13 +3316,13 @@
         <v>2575422.520600178</v>
       </c>
       <c r="D11" t="n">
-        <v>3073461.250099592</v>
+        <v>3073461.250099593</v>
       </c>
       <c r="E11" t="n">
         <v>4177087.695046231</v>
       </c>
       <c r="F11" t="n">
-        <v>6521984.532954988</v>
+        <v>6521984.532954987</v>
       </c>
       <c r="G11" t="n">
         <v>8850627.443805898</v>
@@ -3361,13 +3361,13 @@
         <v>28572353.29459557</v>
       </c>
       <c r="S11" t="n">
-        <v>36088844.77707368</v>
+        <v>36088844.77707367</v>
       </c>
       <c r="T11" t="n">
         <v>44471501.04739226</v>
       </c>
       <c r="U11" t="n">
-        <v>37205495.1415268</v>
+        <v>37205495.14152681</v>
       </c>
       <c r="V11" t="n">
         <v>35680723.44447678</v>
@@ -3384,7 +3384,7 @@
         <v>32698337.55684542</v>
       </c>
       <c r="D12" t="n">
-        <v>42383254.6286003</v>
+        <v>42383254.62860029</v>
       </c>
       <c r="E12" t="n">
         <v>57106524.55837081</v>
@@ -3408,16 +3408,16 @@
         <v>314644743.3356346</v>
       </c>
       <c r="L12" t="n">
-        <v>390346263.7028443</v>
+        <v>390346263.7028444</v>
       </c>
       <c r="M12" t="n">
-        <v>458309314.9543654</v>
+        <v>458309314.9543655</v>
       </c>
       <c r="N12" t="n">
         <v>365494278.16987</v>
       </c>
       <c r="O12" t="n">
-        <v>385179193.7749541</v>
+        <v>385179193.7749543</v>
       </c>
       <c r="P12" t="n">
         <v>343334253.8382795</v>
@@ -3426,7 +3426,7 @@
         <v>384555136.2813308</v>
       </c>
       <c r="R12" t="n">
-        <v>405981632.9934675</v>
+        <v>405981632.9934676</v>
       </c>
       <c r="S12" t="n">
         <v>405387997.9180507</v>
@@ -3438,7 +3438,7 @@
         <v>350395438.5627217</v>
       </c>
       <c r="V12" t="n">
-        <v>352376475.111188</v>
+        <v>352376475.1111879</v>
       </c>
     </row>
     <row r="13">
@@ -3497,7 +3497,7 @@
         <v>85606128.32531728</v>
       </c>
       <c r="S13" t="n">
-        <v>88680507.46830171</v>
+        <v>88680507.4683017</v>
       </c>
       <c r="T13" t="n">
         <v>79947646.57706134</v>
@@ -3535,7 +3535,7 @@
         <v>41949275.6616343</v>
       </c>
       <c r="I14" t="n">
-        <v>54947308.30550973</v>
+        <v>54947308.30550972</v>
       </c>
       <c r="J14" t="n">
         <v>58047872.61953142</v>
@@ -3553,7 +3553,7 @@
         <v>78970352.22843622</v>
       </c>
       <c r="O14" t="n">
-        <v>80387409.64178267</v>
+        <v>80387409.64178266</v>
       </c>
       <c r="P14" t="n">
         <v>80772511.25972682</v>
@@ -3568,13 +3568,13 @@
         <v>69805539.70814623</v>
       </c>
       <c r="T14" t="n">
-        <v>57974078.43708655</v>
+        <v>57974078.43708653</v>
       </c>
       <c r="U14" t="n">
         <v>62014950.08445894</v>
       </c>
       <c r="V14" t="n">
-        <v>80211660.77503592</v>
+        <v>80211660.77503593</v>
       </c>
     </row>
     <row r="15">
@@ -3612,10 +3612,10 @@
         <v>15467815.16656427</v>
       </c>
       <c r="L15" t="n">
-        <v>18016338.81918709</v>
+        <v>18016338.81918708</v>
       </c>
       <c r="M15" t="n">
-        <v>20823121.12731739</v>
+        <v>20823121.1273174</v>
       </c>
       <c r="N15" t="n">
         <v>19164486.76865955</v>
@@ -3624,7 +3624,7 @@
         <v>17763931.62881396</v>
       </c>
       <c r="P15" t="n">
-        <v>19163590.35950671</v>
+        <v>19163590.3595067</v>
       </c>
       <c r="Q15" t="n">
         <v>18356163.83514663</v>
@@ -3660,16 +3660,16 @@
         <v>14361897.08130677</v>
       </c>
       <c r="D16" t="n">
-        <v>20007769.69634736</v>
+        <v>20007769.69634737</v>
       </c>
       <c r="E16" t="n">
-        <v>30685122.23641917</v>
+        <v>30685122.23641916</v>
       </c>
       <c r="F16" t="n">
-        <v>56523301.34897816</v>
+        <v>56523301.34897817</v>
       </c>
       <c r="G16" t="n">
-        <v>81869580.16137905</v>
+        <v>81869580.16137904</v>
       </c>
       <c r="H16" t="n">
         <v>140764654.3436093</v>
@@ -3702,10 +3702,10 @@
         <v>973794179.2776028</v>
       </c>
       <c r="R16" t="n">
-        <v>845216407.065078</v>
+        <v>845216407.0650779</v>
       </c>
       <c r="S16" t="n">
-        <v>983359808.2503392</v>
+        <v>983359808.250339</v>
       </c>
       <c r="T16" t="n">
         <v>1345611369.859587</v>
@@ -3714,7 +3714,7 @@
         <v>1707267436.839567</v>
       </c>
       <c r="V16" t="n">
-        <v>1768293614.169245</v>
+        <v>1768293614.169244</v>
       </c>
     </row>
     <row r="17">
@@ -3725,7 +3725,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>8423660.466274876</v>
+        <v>8423660.466274874</v>
       </c>
       <c r="D17" t="n">
         <v>8811332.059038816</v>
@@ -3761,7 +3761,7 @@
         <v>17823061.44872686</v>
       </c>
       <c r="O17" t="n">
-        <v>15030617.6184825</v>
+        <v>15030617.61848249</v>
       </c>
       <c r="P17" t="n">
         <v>17003047.2480256</v>
@@ -3796,13 +3796,13 @@
         <v>7980607.858265049</v>
       </c>
       <c r="D18" t="n">
-        <v>9150300.211041169</v>
+        <v>9150300.211041166</v>
       </c>
       <c r="E18" t="n">
         <v>10273570.12042056</v>
       </c>
       <c r="F18" t="n">
-        <v>13947661.18916191</v>
+        <v>13947661.18916192</v>
       </c>
       <c r="G18" t="n">
         <v>19240653.22226654</v>
@@ -3814,7 +3814,7 @@
         <v>30139636.77889593</v>
       </c>
       <c r="J18" t="n">
-        <v>28583116.6768156</v>
+        <v>28583116.67681561</v>
       </c>
       <c r="K18" t="n">
         <v>31337987.41436823</v>
@@ -3847,7 +3847,7 @@
         <v>79512741.18478462</v>
       </c>
       <c r="U18" t="n">
-        <v>80483111.75722803</v>
+        <v>80483111.75722805</v>
       </c>
       <c r="V18" t="n">
         <v>83824761.95326656</v>
@@ -3879,7 +3879,7 @@
         <v>621051243.3346971</v>
       </c>
       <c r="I19" t="n">
-        <v>856688038.6987849</v>
+        <v>856688038.6987847</v>
       </c>
       <c r="J19" t="n">
         <v>765091505.8331016</v>
@@ -3903,22 +3903,22 @@
         <v>1880171572.822583</v>
       </c>
       <c r="Q19" t="n">
-        <v>2130578330.495762</v>
+        <v>2130578330.495763</v>
       </c>
       <c r="R19" t="n">
         <v>2812427747.0927</v>
       </c>
       <c r="S19" t="n">
-        <v>2960455583.085769</v>
+        <v>2960455583.085768</v>
       </c>
       <c r="T19" t="n">
-        <v>3132082624.72394</v>
+        <v>3132082624.723941</v>
       </c>
       <c r="U19" t="n">
-        <v>3726700695.924297</v>
+        <v>3726700695.924296</v>
       </c>
       <c r="V19" t="n">
-        <v>3113397475.286286</v>
+        <v>3113397475.286285</v>
       </c>
     </row>
     <row r="20">
@@ -3935,7 +3935,7 @@
         <v>255250938.2078073</v>
       </c>
       <c r="E20" t="n">
-        <v>378235154.3928341</v>
+        <v>378235154.3928339</v>
       </c>
       <c r="F20" t="n">
         <v>461860229.9209856</v>
@@ -3962,16 +3962,16 @@
         <v>1705106131.679287</v>
       </c>
       <c r="N20" t="n">
-        <v>1885389026.083885</v>
+        <v>1885389026.083886</v>
       </c>
       <c r="O20" t="n">
-        <v>3606196899.856905</v>
+        <v>3606196899.856904</v>
       </c>
       <c r="P20" t="n">
         <v>4013951531.518703</v>
       </c>
       <c r="Q20" t="n">
-        <v>3634772952.775167</v>
+        <v>3634772952.775168</v>
       </c>
       <c r="R20" t="n">
         <v>3294839503.3944</v>
@@ -3980,7 +3980,7 @@
         <v>3337939484.596141</v>
       </c>
       <c r="T20" t="n">
-        <v>4195064492.505627</v>
+        <v>4195064492.505628</v>
       </c>
       <c r="U20" t="n">
         <v>4306312842.737441</v>
@@ -3997,10 +3997,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>55765360.63328119</v>
+        <v>55765360.6332812</v>
       </c>
       <c r="D21" t="n">
-        <v>69632020.91142011</v>
+        <v>69632020.91142009</v>
       </c>
       <c r="E21" t="n">
         <v>81663935.15774971</v>
@@ -4030,13 +4030,13 @@
         <v>660120971.3052415</v>
       </c>
       <c r="N21" t="n">
-        <v>738118429.7179865</v>
+        <v>738118429.7179866</v>
       </c>
       <c r="O21" t="n">
-        <v>719830030.1044499</v>
+        <v>719830030.1044497</v>
       </c>
       <c r="P21" t="n">
-        <v>656399816.6915035</v>
+        <v>656399816.6915036</v>
       </c>
       <c r="Q21" t="n">
         <v>664427131.2677928</v>
@@ -4045,7 +4045,7 @@
         <v>702232216.8749601</v>
       </c>
       <c r="S21" t="n">
-        <v>638983887.7944446</v>
+        <v>638983887.7944444</v>
       </c>
       <c r="T21" t="n">
         <v>765950211.621523</v>
@@ -4054,7 +4054,7 @@
         <v>860377199.7310314</v>
       </c>
       <c r="V21" t="n">
-        <v>844644893.5636971</v>
+        <v>844644893.563697</v>
       </c>
     </row>
     <row r="22">
@@ -4075,7 +4075,7 @@
         <v>3370859.835794372</v>
       </c>
       <c r="E22" t="n">
-        <v>5281976.965276654</v>
+        <v>5281976.965276653</v>
       </c>
       <c r="F22" t="n">
         <v>2176830.905548199</v>
@@ -4105,10 +4105,10 @@
         <v>51181348.98379238</v>
       </c>
       <c r="O22" t="n">
-        <v>55931803.14252406</v>
+        <v>55931803.14252405</v>
       </c>
       <c r="P22" t="n">
-        <v>39364721.41177321</v>
+        <v>39364721.4117732</v>
       </c>
       <c r="Q22" t="n">
         <v>37900947.39546846</v>
@@ -4126,7 +4126,7 @@
         <v>59575098.94340524</v>
       </c>
       <c r="V22" t="n">
-        <v>53422120.96544281</v>
+        <v>53422120.96544278</v>
       </c>
     </row>
     <row r="23">
@@ -4173,7 +4173,7 @@
         <v>296508080.6930175</v>
       </c>
       <c r="O23" t="n">
-        <v>303304146.7370696</v>
+        <v>303304146.7370695</v>
       </c>
       <c r="P23" t="n">
         <v>325352623.8292806</v>
@@ -4191,7 +4191,7 @@
         <v>586445047.493422</v>
       </c>
       <c r="U23" t="n">
-        <v>610196045.7879744</v>
+        <v>610196045.7879742</v>
       </c>
       <c r="V23" t="n">
         <v>693543686.2218848</v>
@@ -4235,7 +4235,7 @@
         <v>16498959.74382464</v>
       </c>
       <c r="M24" t="n">
-        <v>30098817.26442954</v>
+        <v>30098817.26442953</v>
       </c>
       <c r="N24" t="n">
         <v>40201549.82422977</v>
@@ -4244,7 +4244,7 @@
         <v>37385874.31143112</v>
       </c>
       <c r="P24" t="n">
-        <v>33854860.11508892</v>
+        <v>33854860.11508891</v>
       </c>
       <c r="Q24" t="n">
         <v>39361769.03859016</v>
@@ -4262,7 +4262,7 @@
         <v>74330494.44362603</v>
       </c>
       <c r="V24" t="n">
-        <v>88384897.9512998</v>
+        <v>88384897.95129982</v>
       </c>
     </row>
     <row r="25">
@@ -4279,7 +4279,7 @@
         <v>366.3649762696028</v>
       </c>
       <c r="E25" t="n">
-        <v>88194.97803190048</v>
+        <v>88194.97803190049</v>
       </c>
       <c r="F25" t="n">
         <v>183776.9472670676</v>
@@ -4297,7 +4297,7 @@
         <v>2261292.634534216</v>
       </c>
       <c r="K25" t="n">
-        <v>2636309.42368848</v>
+        <v>2636309.423688481</v>
       </c>
       <c r="L25" t="n">
         <v>3482821.84057851</v>
@@ -4321,7 +4321,7 @@
         <v>8515265.423207151</v>
       </c>
       <c r="S25" t="n">
-        <v>7009532.534379893</v>
+        <v>7009532.534379894</v>
       </c>
       <c r="T25" t="n">
         <v>8777923.048372375</v>
@@ -4341,13 +4341,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3458622.428447074</v>
+        <v>3458622.428447075</v>
       </c>
       <c r="D26" t="n">
         <v>4513979.834222752</v>
       </c>
       <c r="E26" t="n">
-        <v>7373094.603773806</v>
+        <v>7373094.603773808</v>
       </c>
       <c r="F26" t="n">
         <v>9572741.46547796</v>
@@ -4362,7 +4362,7 @@
         <v>31414608.96122916</v>
       </c>
       <c r="J26" t="n">
-        <v>31624589.90528526</v>
+        <v>31624589.90528525</v>
       </c>
       <c r="K26" t="n">
         <v>42889341.85882319</v>
@@ -4374,13 +4374,13 @@
         <v>54898631.16124289</v>
       </c>
       <c r="N26" t="n">
-        <v>69314434.95163929</v>
+        <v>69314434.95163931</v>
       </c>
       <c r="O26" t="n">
         <v>93170636.29838063</v>
       </c>
       <c r="P26" t="n">
-        <v>92343067.17484091</v>
+        <v>92343067.17484093</v>
       </c>
       <c r="Q26" t="n">
         <v>91747589.36044668</v>
@@ -4392,7 +4392,7 @@
         <v>264169655.5397286</v>
       </c>
       <c r="T26" t="n">
-        <v>81800808.39466716</v>
+        <v>81800808.39466713</v>
       </c>
       <c r="U26" t="n">
         <v>74664168.16061009</v>
@@ -4422,7 +4422,7 @@
         <v>1941304.965021861</v>
       </c>
       <c r="F27" t="n">
-        <v>4799933.713529073</v>
+        <v>4799933.713529074</v>
       </c>
       <c r="G27" t="n">
         <v>4915398.534991422</v>
@@ -4437,22 +4437,22 @@
         <v>13529024.36035665</v>
       </c>
       <c r="K27" t="n">
-        <v>23327402.89741363</v>
+        <v>23327402.89741364</v>
       </c>
       <c r="L27" t="n">
         <v>28439994.32114946</v>
       </c>
       <c r="M27" t="n">
-        <v>36960523.28463062</v>
+        <v>36960523.28463063</v>
       </c>
       <c r="N27" t="n">
-        <v>40189135.29030263</v>
+        <v>40189135.29030264</v>
       </c>
       <c r="O27" t="n">
         <v>46764683.44621938</v>
       </c>
       <c r="P27" t="n">
-        <v>44237035.94041079</v>
+        <v>44237035.94041078</v>
       </c>
       <c r="Q27" t="n">
         <v>47420721.23194028</v>
@@ -4461,13 +4461,13 @@
         <v>47908415.82176396</v>
       </c>
       <c r="S27" t="n">
-        <v>59528334.93329747</v>
+        <v>59528334.93329746</v>
       </c>
       <c r="T27" t="n">
-        <v>68678003.20389356</v>
+        <v>68678003.20389359</v>
       </c>
       <c r="U27" t="n">
-        <v>76235436.30376063</v>
+        <v>76235436.30376062</v>
       </c>
       <c r="V27" t="n">
         <v>86203636.65401636</v>
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9406455.978975726</v>
+        <v>9406455.978975724</v>
       </c>
       <c r="D28" t="n">
         <v>10655470.98510596</v>
@@ -4529,7 +4529,7 @@
         <v>264811408.2682282</v>
       </c>
       <c r="S28" t="n">
-        <v>301773788.4928433</v>
+        <v>301773788.4928434</v>
       </c>
       <c r="T28" t="n">
         <v>349028049.671914</v>
@@ -4552,7 +4552,7 @@
         <v>5662886.837364792</v>
       </c>
       <c r="D29" t="n">
-        <v>7263275.891740758</v>
+        <v>7263275.891740755</v>
       </c>
       <c r="E29" t="n">
         <v>9044958.818462802</v>
@@ -4576,7 +4576,7 @@
         <v>26463460.27073513</v>
       </c>
       <c r="L29" t="n">
-        <v>28528506.57952982</v>
+        <v>28528506.57952983</v>
       </c>
       <c r="M29" t="n">
         <v>35224742.9229902</v>
@@ -4588,16 +4588,16 @@
         <v>51713644.19038891</v>
       </c>
       <c r="P29" t="n">
-        <v>58164728.17663568</v>
+        <v>58164728.17663569</v>
       </c>
       <c r="Q29" t="n">
         <v>37162007.42133451</v>
       </c>
       <c r="R29" t="n">
-        <v>33556776.0802834</v>
+        <v>33556776.08028341</v>
       </c>
       <c r="S29" t="n">
-        <v>39615294.7335697</v>
+        <v>39615294.73356971</v>
       </c>
       <c r="T29" t="n">
         <v>38045034.22474975</v>
@@ -4635,10 +4635,10 @@
         <v>61273859.82986093</v>
       </c>
       <c r="I30" t="n">
-        <v>84517577.95449889</v>
+        <v>84517577.95449892</v>
       </c>
       <c r="J30" t="n">
-        <v>106166167.5475831</v>
+        <v>106166167.547583</v>
       </c>
       <c r="K30" t="n">
         <v>138817466.984978</v>
@@ -4653,7 +4653,7 @@
         <v>377535948.9645351</v>
       </c>
       <c r="O30" t="n">
-        <v>486240573.8744697</v>
+        <v>486240573.8744698</v>
       </c>
       <c r="P30" t="n">
         <v>515035888.2898036</v>
@@ -4668,13 +4668,13 @@
         <v>805685496.6359696</v>
       </c>
       <c r="T30" t="n">
-        <v>761689073.6513082</v>
+        <v>761689073.6513081</v>
       </c>
       <c r="U30" t="n">
         <v>891596027.4886978</v>
       </c>
       <c r="V30" t="n">
-        <v>870527314.9061463</v>
+        <v>870527314.9061462</v>
       </c>
     </row>
     <row r="31">
@@ -4691,16 +4691,16 @@
         <v>161178.3965757757</v>
       </c>
       <c r="E31" t="n">
-        <v>199002.4600456683</v>
+        <v>199002.4600456682</v>
       </c>
       <c r="F31" t="n">
-        <v>223525.0388296549</v>
+        <v>223525.0388296548</v>
       </c>
       <c r="G31" t="n">
         <v>284494.9162113282</v>
       </c>
       <c r="H31" t="n">
-        <v>612427.5370858565</v>
+        <v>612427.5370858568</v>
       </c>
       <c r="I31" t="n">
         <v>831124.8998762243</v>
@@ -4718,7 +4718,7 @@
         <v>3288218.675184585</v>
       </c>
       <c r="N31" t="n">
-        <v>4322475.247774466</v>
+        <v>4322475.247774467</v>
       </c>
       <c r="O31" t="n">
         <v>6034928.00114781</v>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7297551.865734555</v>
+        <v>7297551.865734553</v>
       </c>
       <c r="D2" t="n">
         <v>8109509.929190547</v>
@@ -4866,19 +4866,19 @@
         <v>19726576.50695829</v>
       </c>
       <c r="H2" t="n">
-        <v>28248335.29420202</v>
+        <v>28248335.29420203</v>
       </c>
       <c r="I2" t="n">
         <v>32536577.09778854</v>
       </c>
       <c r="J2" t="n">
-        <v>32658875.52211106</v>
+        <v>32658875.52211107</v>
       </c>
       <c r="K2" t="n">
         <v>34143679.92372525</v>
       </c>
       <c r="L2" t="n">
-        <v>39798416.80747766</v>
+        <v>39798416.80747765</v>
       </c>
       <c r="M2" t="n">
         <v>52514620.97976325</v>
@@ -4893,16 +4893,16 @@
         <v>48162399.99612322</v>
       </c>
       <c r="Q2" t="n">
-        <v>44724890.90538349</v>
+        <v>44724890.9053835</v>
       </c>
       <c r="R2" t="n">
-        <v>42923240.19080244</v>
+        <v>42923240.19080245</v>
       </c>
       <c r="S2" t="n">
-        <v>44456324.98694749</v>
+        <v>44456324.98694748</v>
       </c>
       <c r="T2" t="n">
-        <v>37207758.26577729</v>
+        <v>37207758.26577728</v>
       </c>
       <c r="U2" t="n">
         <v>39225212.25101089</v>
@@ -4919,16 +4919,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>77338315.29440458</v>
+        <v>77338315.2944046</v>
       </c>
       <c r="D3" t="n">
         <v>86637800.38308369</v>
       </c>
       <c r="E3" t="n">
-        <v>97177216.09154342</v>
+        <v>97177216.09154341</v>
       </c>
       <c r="F3" t="n">
-        <v>117898883.9953371</v>
+        <v>117898883.9953372</v>
       </c>
       <c r="G3" t="n">
         <v>132549738.4015062</v>
@@ -4958,13 +4958,13 @@
         <v>377035116.5146663</v>
       </c>
       <c r="P3" t="n">
-        <v>398264885.1953276</v>
+        <v>398264885.1953277</v>
       </c>
       <c r="Q3" t="n">
-        <v>388554948.9349984</v>
+        <v>388554948.9349983</v>
       </c>
       <c r="R3" t="n">
-        <v>408711583.8488938</v>
+        <v>408711583.8488936</v>
       </c>
       <c r="S3" t="n">
         <v>466408810.6086047</v>
@@ -4987,13 +4987,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>31306875.41377294</v>
+        <v>31306875.41377295</v>
       </c>
       <c r="D4" t="n">
-        <v>32224200.04152193</v>
+        <v>32224200.04152194</v>
       </c>
       <c r="E4" t="n">
-        <v>38058945.89327795</v>
+        <v>38058945.89327794</v>
       </c>
       <c r="F4" t="n">
         <v>44387415.18005716</v>
@@ -5014,7 +5014,7 @@
         <v>80528168.5612801</v>
       </c>
       <c r="L4" t="n">
-        <v>84331098.03805807</v>
+        <v>84331098.03805809</v>
       </c>
       <c r="M4" t="n">
         <v>111990815.7972604</v>
@@ -5080,10 +5080,10 @@
         <v>79100985.07517616</v>
       </c>
       <c r="J5" t="n">
-        <v>76018227.67319052</v>
+        <v>76018227.6731905</v>
       </c>
       <c r="K5" t="n">
-        <v>77363687.9182788</v>
+        <v>77363687.91827881</v>
       </c>
       <c r="L5" t="n">
         <v>91183431.43160114</v>
@@ -5145,7 +5145,7 @@
         <v>33911396.84626037</v>
       </c>
       <c r="I6" t="n">
-        <v>37839250.16014289</v>
+        <v>37839250.16014288</v>
       </c>
       <c r="J6" t="n">
         <v>43455259.12962165</v>
@@ -5163,7 +5163,7 @@
         <v>79444538.93989263</v>
       </c>
       <c r="O6" t="n">
-        <v>96552455.97946303</v>
+        <v>96552455.97946301</v>
       </c>
       <c r="P6" t="n">
         <v>104649710.9397986</v>
@@ -5178,7 +5178,7 @@
         <v>133288456.8756433</v>
       </c>
       <c r="T6" t="n">
-        <v>136007088.1871907</v>
+        <v>136007088.1871908</v>
       </c>
       <c r="U6" t="n">
         <v>134607626.6576061</v>
@@ -5213,7 +5213,7 @@
         <v>174958997.155363</v>
       </c>
       <c r="I7" t="n">
-        <v>208673396.3142149</v>
+        <v>208673396.3142148</v>
       </c>
       <c r="J7" t="n">
         <v>233882109.804249</v>
@@ -5231,13 +5231,13 @@
         <v>447036552.0634882</v>
       </c>
       <c r="O7" t="n">
-        <v>493289309.0114428</v>
+        <v>493289309.011443</v>
       </c>
       <c r="P7" t="n">
         <v>522261928.8363445</v>
       </c>
       <c r="Q7" t="n">
-        <v>613483368.812398</v>
+        <v>613483368.8123981</v>
       </c>
       <c r="R7" t="n">
         <v>664982194.6400687</v>
@@ -5246,13 +5246,13 @@
         <v>720798327.1863563</v>
       </c>
       <c r="T7" t="n">
-        <v>711340967.3433592</v>
+        <v>711340967.3433594</v>
       </c>
       <c r="U7" t="n">
-        <v>816077119.5402864</v>
+        <v>816077119.5402865</v>
       </c>
       <c r="V7" t="n">
-        <v>810533467.723121</v>
+        <v>810533467.7231209</v>
       </c>
     </row>
     <row r="8">
@@ -5272,7 +5272,7 @@
         <v>30112345.54382956</v>
       </c>
       <c r="F8" t="n">
-        <v>42723634.96973796</v>
+        <v>42723634.96973797</v>
       </c>
       <c r="G8" t="n">
         <v>61610738.88777693</v>
@@ -5290,13 +5290,13 @@
         <v>122644711.0751429</v>
       </c>
       <c r="L8" t="n">
-        <v>138605491.076623</v>
+        <v>138605491.0766229</v>
       </c>
       <c r="M8" t="n">
         <v>161196852.7938213</v>
       </c>
       <c r="N8" t="n">
-        <v>167719330.585362</v>
+        <v>167719330.5853621</v>
       </c>
       <c r="O8" t="n">
         <v>179640211.6329705</v>
@@ -5314,13 +5314,13 @@
         <v>243487593.4221445</v>
       </c>
       <c r="T8" t="n">
-        <v>246221006.5052282</v>
+        <v>246221006.5052281</v>
       </c>
       <c r="U8" t="n">
-        <v>264847673.6136711</v>
+        <v>264847673.6136712</v>
       </c>
       <c r="V8" t="n">
-        <v>312461988.2480982</v>
+        <v>312461988.2480983</v>
       </c>
     </row>
     <row r="9">
@@ -5361,10 +5361,10 @@
         <v>38679773.52761649</v>
       </c>
       <c r="M9" t="n">
-        <v>45717351.11468266</v>
+        <v>45717351.11468267</v>
       </c>
       <c r="N9" t="n">
-        <v>47858854.44750314</v>
+        <v>47858854.44750315</v>
       </c>
       <c r="O9" t="n">
         <v>47188280.56466439</v>
@@ -5376,16 +5376,16 @@
         <v>62714603.06305638</v>
       </c>
       <c r="R9" t="n">
-        <v>61272723.40413925</v>
+        <v>61272723.40413924</v>
       </c>
       <c r="S9" t="n">
-        <v>71241931.76851395</v>
+        <v>71241931.76851396</v>
       </c>
       <c r="T9" t="n">
         <v>79405613.22522503</v>
       </c>
       <c r="U9" t="n">
-        <v>96611535.91360192</v>
+        <v>96611535.91360191</v>
       </c>
       <c r="V9" t="n">
         <v>93942101.61745349</v>
@@ -5409,10 +5409,10 @@
         <v>15897903.08540693</v>
       </c>
       <c r="E10" t="n">
-        <v>23556984.62847036</v>
+        <v>23556984.62847037</v>
       </c>
       <c r="F10" t="n">
-        <v>34271817.91142778</v>
+        <v>34271817.91142779</v>
       </c>
       <c r="G10" t="n">
         <v>32644677.90575694</v>
@@ -5424,7 +5424,7 @@
         <v>64417343.4497679</v>
       </c>
       <c r="J10" t="n">
-        <v>74522947.65262936</v>
+        <v>74522947.65262938</v>
       </c>
       <c r="K10" t="n">
         <v>99516166.48769748</v>
@@ -5436,22 +5436,22 @@
         <v>139853416.1789991</v>
       </c>
       <c r="N10" t="n">
-        <v>165687938.4292055</v>
+        <v>165687938.4292054</v>
       </c>
       <c r="O10" t="n">
         <v>180533529.0417282</v>
       </c>
       <c r="P10" t="n">
-        <v>205458281.0599209</v>
+        <v>205458281.0599208</v>
       </c>
       <c r="Q10" t="n">
         <v>202505866.9300326</v>
       </c>
       <c r="R10" t="n">
-        <v>216340952.0564095</v>
+        <v>216340952.0564094</v>
       </c>
       <c r="S10" t="n">
-        <v>299588881.5591364</v>
+        <v>299588881.5591363</v>
       </c>
       <c r="T10" t="n">
         <v>163169165.1344512</v>
@@ -5477,7 +5477,7 @@
         <v>3629534.396467749</v>
       </c>
       <c r="E11" t="n">
-        <v>4835001.330208036</v>
+        <v>4835001.330208035</v>
       </c>
       <c r="F11" t="n">
         <v>6241401.299336469</v>
@@ -5492,7 +5492,7 @@
         <v>15275991.78561078</v>
       </c>
       <c r="J11" t="n">
-        <v>15854863.17752919</v>
+        <v>15854863.17752918</v>
       </c>
       <c r="K11" t="n">
         <v>19484539.85540636</v>
@@ -5510,7 +5510,7 @@
         <v>31790802.62615632</v>
       </c>
       <c r="P11" t="n">
-        <v>33092025.8552179</v>
+        <v>33092025.85521791</v>
       </c>
       <c r="Q11" t="n">
         <v>35655052.98097502</v>
@@ -5522,7 +5522,7 @@
         <v>41829585.04580639</v>
       </c>
       <c r="T11" t="n">
-        <v>45509635.01021258</v>
+        <v>45509635.01021259</v>
       </c>
       <c r="U11" t="n">
         <v>46704421.6661284</v>
@@ -5539,7 +5539,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30493248.46800504</v>
+        <v>30493248.46800505</v>
       </c>
       <c r="D12" t="n">
         <v>34980899.73859484</v>
@@ -5557,7 +5557,7 @@
         <v>147440299.9251099</v>
       </c>
       <c r="I12" t="n">
-        <v>179999649.356521</v>
+        <v>179999649.3565209</v>
       </c>
       <c r="J12" t="n">
         <v>182575672.7344544</v>
@@ -5566,7 +5566,7 @@
         <v>226697640.1053773</v>
       </c>
       <c r="L12" t="n">
-        <v>274576394.3857555</v>
+        <v>274576394.3857556</v>
       </c>
       <c r="M12" t="n">
         <v>327374733.3485788</v>
@@ -5584,7 +5584,7 @@
         <v>301215535.5359043</v>
       </c>
       <c r="R12" t="n">
-        <v>320268296.1517469</v>
+        <v>320268296.151747</v>
       </c>
       <c r="S12" t="n">
         <v>322834734.030315</v>
@@ -5593,7 +5593,7 @@
         <v>290245123.4092836</v>
       </c>
       <c r="U12" t="n">
-        <v>293360463.2837391</v>
+        <v>293360463.2837392</v>
       </c>
       <c r="V12" t="n">
         <v>305143747.4212378</v>
@@ -5619,7 +5619,7 @@
         <v>27015387.42959125</v>
       </c>
       <c r="G13" t="n">
-        <v>36112627.22416678</v>
+        <v>36112627.22416679</v>
       </c>
       <c r="H13" t="n">
         <v>49892306.45086109</v>
@@ -5631,10 +5631,10 @@
         <v>70184963.87011702</v>
       </c>
       <c r="K13" t="n">
-        <v>81723228.36157568</v>
+        <v>81723228.36157566</v>
       </c>
       <c r="L13" t="n">
-        <v>93666358.34021632</v>
+        <v>93666358.34021634</v>
       </c>
       <c r="M13" t="n">
         <v>114327613.5443233</v>
@@ -5661,10 +5661,10 @@
         <v>121444257.7146107</v>
       </c>
       <c r="U13" t="n">
-        <v>133468209.3684226</v>
+        <v>133468209.3684225</v>
       </c>
       <c r="V13" t="n">
-        <v>143819785.1461363</v>
+        <v>143819785.1461364</v>
       </c>
     </row>
     <row r="14">
@@ -5687,19 +5687,19 @@
         <v>17223391.30278577</v>
       </c>
       <c r="G14" t="n">
-        <v>35891255.00705616</v>
+        <v>35891255.00705615</v>
       </c>
       <c r="H14" t="n">
         <v>53074212.26522493</v>
       </c>
       <c r="I14" t="n">
-        <v>65459075.20728936</v>
+        <v>65459075.20728938</v>
       </c>
       <c r="J14" t="n">
         <v>79769627.75482538</v>
       </c>
       <c r="K14" t="n">
-        <v>99135264.60203718</v>
+        <v>99135264.60203716</v>
       </c>
       <c r="L14" t="n">
         <v>106640947.9125495</v>
@@ -5726,7 +5726,7 @@
         <v>102760741.3761516</v>
       </c>
       <c r="T14" t="n">
-        <v>93729270.00417924</v>
+        <v>93729270.00417922</v>
       </c>
       <c r="U14" t="n">
         <v>100506518.9852943</v>
@@ -5758,7 +5758,7 @@
         <v>7402921.393444247</v>
       </c>
       <c r="H15" t="n">
-        <v>9914428.343339356</v>
+        <v>9914428.343339359</v>
       </c>
       <c r="I15" t="n">
         <v>12405439.93677728</v>
@@ -5773,16 +5773,16 @@
         <v>31188659.41659281</v>
       </c>
       <c r="M15" t="n">
-        <v>33989788.66110138</v>
+        <v>33989788.66110139</v>
       </c>
       <c r="N15" t="n">
-        <v>36140763.17421915</v>
+        <v>36140763.17421916</v>
       </c>
       <c r="O15" t="n">
         <v>26827074.12709973</v>
       </c>
       <c r="P15" t="n">
-        <v>33905055.5222169</v>
+        <v>33905055.52221691</v>
       </c>
       <c r="Q15" t="n">
         <v>35165991.03204939</v>
@@ -5827,10 +5827,10 @@
         <v>50073708.73015305</v>
       </c>
       <c r="G16" t="n">
-        <v>66224294.85323212</v>
+        <v>66224294.85323213</v>
       </c>
       <c r="H16" t="n">
-        <v>95018197.68608727</v>
+        <v>95018197.68608724</v>
       </c>
       <c r="I16" t="n">
         <v>132561546.1483248</v>
@@ -5851,10 +5851,10 @@
         <v>520325411.411096</v>
       </c>
       <c r="O16" t="n">
-        <v>527429696.2000068</v>
+        <v>527429696.2000067</v>
       </c>
       <c r="P16" t="n">
-        <v>532800305.0717223</v>
+        <v>532800305.0717222</v>
       </c>
       <c r="Q16" t="n">
         <v>503977115.7348011</v>
@@ -5866,13 +5866,13 @@
         <v>553082378.9600302</v>
       </c>
       <c r="T16" t="n">
-        <v>713087573.2325839</v>
+        <v>713087573.2325838</v>
       </c>
       <c r="U16" t="n">
-        <v>851310416.2630247</v>
+        <v>851310416.2630246</v>
       </c>
       <c r="V16" t="n">
-        <v>895244635.9562573</v>
+        <v>895244635.9562576</v>
       </c>
     </row>
     <row r="17">
@@ -5913,13 +5913,13 @@
         <v>24446900.18455883</v>
       </c>
       <c r="M17" t="n">
-        <v>23257261.24846112</v>
+        <v>23257261.24846111</v>
       </c>
       <c r="N17" t="n">
         <v>24795462.5222609</v>
       </c>
       <c r="O17" t="n">
-        <v>21719774.24266129</v>
+        <v>21719774.24266128</v>
       </c>
       <c r="P17" t="n">
         <v>22934297.1296826</v>
@@ -5940,7 +5940,7 @@
         <v>31347611.86337438</v>
       </c>
       <c r="V17" t="n">
-        <v>24899586.44499984</v>
+        <v>24899586.44499985</v>
       </c>
     </row>
     <row r="18">
@@ -5951,7 +5951,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>7525677.584631672</v>
+        <v>7525677.584631671</v>
       </c>
       <c r="D18" t="n">
         <v>8816622.988257904</v>
@@ -5966,10 +5966,10 @@
         <v>17745132.3067802</v>
       </c>
       <c r="H18" t="n">
-        <v>23135103.16591723</v>
+        <v>23135103.16591724</v>
       </c>
       <c r="I18" t="n">
-        <v>25710608.67826095</v>
+        <v>25710608.67826096</v>
       </c>
       <c r="J18" t="n">
         <v>30338899.11514191</v>
@@ -5990,10 +5990,10 @@
         <v>74054649.47100353</v>
       </c>
       <c r="P18" t="n">
-        <v>75889318.84252763</v>
+        <v>75889318.84252761</v>
       </c>
       <c r="Q18" t="n">
-        <v>79501402.75207081</v>
+        <v>79501402.75207083</v>
       </c>
       <c r="R18" t="n">
         <v>81185555.87418899</v>
@@ -6002,13 +6002,13 @@
         <v>71225966.45261301</v>
       </c>
       <c r="T18" t="n">
-        <v>72645369.35160251</v>
+        <v>72645369.35160252</v>
       </c>
       <c r="U18" t="n">
         <v>77609697.34575391</v>
       </c>
       <c r="V18" t="n">
-        <v>81704818.17263505</v>
+        <v>81704818.17263503</v>
       </c>
     </row>
     <row r="19">
@@ -6034,28 +6034,28 @@
         <v>313762960.9707202</v>
       </c>
       <c r="H19" t="n">
-        <v>420463470.1770359</v>
+        <v>420463470.1770357</v>
       </c>
       <c r="I19" t="n">
         <v>537863136.6388208</v>
       </c>
       <c r="J19" t="n">
-        <v>572046502.9692906</v>
+        <v>572046502.9692907</v>
       </c>
       <c r="K19" t="n">
-        <v>638953121.6347188</v>
+        <v>638953121.6347187</v>
       </c>
       <c r="L19" t="n">
         <v>782703684.0939964</v>
       </c>
       <c r="M19" t="n">
-        <v>892122842.9696904</v>
+        <v>892122842.9696907</v>
       </c>
       <c r="N19" t="n">
         <v>989297926.2004344</v>
       </c>
       <c r="O19" t="n">
-        <v>974383060.2250843</v>
+        <v>974383060.2250844</v>
       </c>
       <c r="P19" t="n">
         <v>1073267559.523186</v>
@@ -6067,10 +6067,10 @@
         <v>1220916311.593204</v>
       </c>
       <c r="S19" t="n">
-        <v>1295163350.430797</v>
+        <v>1295163350.430796</v>
       </c>
       <c r="T19" t="n">
-        <v>1437285857.755604</v>
+        <v>1437285857.755603</v>
       </c>
       <c r="U19" t="n">
         <v>1676279626.236734</v>
@@ -6090,10 +6090,10 @@
         <v>79412568.72685468</v>
       </c>
       <c r="D20" t="n">
-        <v>118696452.1970865</v>
+        <v>118696452.1970864</v>
       </c>
       <c r="E20" t="n">
-        <v>151695786.4455614</v>
+        <v>151695786.4455615</v>
       </c>
       <c r="F20" t="n">
         <v>189102007.2130735</v>
@@ -6105,7 +6105,7 @@
         <v>304495775.0834427</v>
       </c>
       <c r="I20" t="n">
-        <v>369182891.9208569</v>
+        <v>369182891.9208568</v>
       </c>
       <c r="J20" t="n">
         <v>409919264.0758414</v>
@@ -6117,28 +6117,28 @@
         <v>428817961.7465392</v>
       </c>
       <c r="M20" t="n">
-        <v>515590977.7277243</v>
+        <v>515590977.7277242</v>
       </c>
       <c r="N20" t="n">
         <v>568446491.9055427</v>
       </c>
       <c r="O20" t="n">
-        <v>763632658.1940101</v>
+        <v>763632658.1940103</v>
       </c>
       <c r="P20" t="n">
-        <v>790869930.1511849</v>
+        <v>790869930.151185</v>
       </c>
       <c r="Q20" t="n">
         <v>742649167.0278795</v>
       </c>
       <c r="R20" t="n">
-        <v>702690670.3436812</v>
+        <v>702690670.3436813</v>
       </c>
       <c r="S20" t="n">
         <v>736013596.8577054</v>
       </c>
       <c r="T20" t="n">
-        <v>809406746.4606651</v>
+        <v>809406746.4606652</v>
       </c>
       <c r="U20" t="n">
         <v>872991020.2817374</v>
@@ -6155,13 +6155,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>56051295.73681355</v>
+        <v>56051295.73681354</v>
       </c>
       <c r="D21" t="n">
-        <v>68073749.1280061</v>
+        <v>68073749.12800612</v>
       </c>
       <c r="E21" t="n">
-        <v>87819149.973979</v>
+        <v>87819149.97397903</v>
       </c>
       <c r="F21" t="n">
         <v>121004398.7909041</v>
@@ -6185,13 +6185,13 @@
         <v>431533146.9613695</v>
       </c>
       <c r="M21" t="n">
-        <v>540675959.4024527</v>
+        <v>540675959.4024526</v>
       </c>
       <c r="N21" t="n">
-        <v>635561875.5137153</v>
+        <v>635561875.5137151</v>
       </c>
       <c r="O21" t="n">
-        <v>612796278.7847995</v>
+        <v>612796278.7847993</v>
       </c>
       <c r="P21" t="n">
         <v>568789278.0422486</v>
@@ -6203,13 +6203,13 @@
         <v>634194864.8251292</v>
       </c>
       <c r="S21" t="n">
-        <v>608186995.4364067</v>
+        <v>608186995.4364066</v>
       </c>
       <c r="T21" t="n">
-        <v>774512287.6339895</v>
+        <v>774512287.6339896</v>
       </c>
       <c r="U21" t="n">
-        <v>796257986.6467105</v>
+        <v>796257986.6467104</v>
       </c>
       <c r="V21" t="n">
         <v>837113482.7278769</v>
@@ -6227,13 +6227,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4002836.52278346</v>
+        <v>4002836.522783461</v>
       </c>
       <c r="D22" t="n">
-        <v>5222952.695726843</v>
+        <v>5222952.695726844</v>
       </c>
       <c r="E22" t="n">
-        <v>7459012.866514144</v>
+        <v>7459012.866514146</v>
       </c>
       <c r="F22" t="n">
         <v>3743695.850699771</v>
@@ -6257,16 +6257,16 @@
         <v>39304167.3817085</v>
       </c>
       <c r="M22" t="n">
-        <v>43376945.61435025</v>
+        <v>43376945.61435024</v>
       </c>
       <c r="N22" t="n">
-        <v>55162880.0164033</v>
+        <v>55162880.01640329</v>
       </c>
       <c r="O22" t="n">
-        <v>56707569.17943067</v>
+        <v>56707569.17943066</v>
       </c>
       <c r="P22" t="n">
-        <v>50664415.20718377</v>
+        <v>50664415.20718378</v>
       </c>
       <c r="Q22" t="n">
         <v>50654165.78527138</v>
@@ -6278,13 +6278,13 @@
         <v>58175140.12187527</v>
       </c>
       <c r="T22" t="n">
-        <v>70027650.20629929</v>
+        <v>70027650.20629928</v>
       </c>
       <c r="U22" t="n">
         <v>80707464.27873735</v>
       </c>
       <c r="V22" t="n">
-        <v>81838031.70058535</v>
+        <v>81838031.70058537</v>
       </c>
     </row>
     <row r="23">
@@ -6307,7 +6307,7 @@
         <v>102083606.9269855</v>
       </c>
       <c r="G23" t="n">
-        <v>124329506.0700151</v>
+        <v>124329506.0700152</v>
       </c>
       <c r="H23" t="n">
         <v>176660074.4223381</v>
@@ -6343,13 +6343,13 @@
         <v>221834792.7416061</v>
       </c>
       <c r="S23" t="n">
-        <v>520502719.641529</v>
+        <v>520502719.6415291</v>
       </c>
       <c r="T23" t="n">
         <v>567581712.8379471</v>
       </c>
       <c r="U23" t="n">
-        <v>599423851.9005998</v>
+        <v>599423851.9006</v>
       </c>
       <c r="V23" t="n">
         <v>633148737.8640012</v>
@@ -6375,13 +6375,13 @@
         <v>7022890.469590347</v>
       </c>
       <c r="G24" t="n">
-        <v>9329931.661485834</v>
+        <v>9329931.661485836</v>
       </c>
       <c r="H24" t="n">
         <v>12689884.05653313</v>
       </c>
       <c r="I24" t="n">
-        <v>17494611.47108466</v>
+        <v>17494611.47108467</v>
       </c>
       <c r="J24" t="n">
         <v>18080496.1774699</v>
@@ -6399,19 +6399,19 @@
         <v>46336157.28616322</v>
       </c>
       <c r="O24" t="n">
-        <v>42595006.41869983</v>
+        <v>42595006.41869984</v>
       </c>
       <c r="P24" t="n">
-        <v>44530842.30014286</v>
+        <v>44530842.30014285</v>
       </c>
       <c r="Q24" t="n">
         <v>49865481.58942378</v>
       </c>
       <c r="R24" t="n">
-        <v>48642635.85754445</v>
+        <v>48642635.85754444</v>
       </c>
       <c r="S24" t="n">
-        <v>55693158.08279008</v>
+        <v>55693158.08279007</v>
       </c>
       <c r="T24" t="n">
         <v>55945577.44746925</v>
@@ -6420,7 +6420,7 @@
         <v>73835342.31833853</v>
       </c>
       <c r="V24" t="n">
-        <v>86839717.57266568</v>
+        <v>86839717.57266566</v>
       </c>
     </row>
     <row r="25">
@@ -6431,13 +6431,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>82448.76623670527</v>
+        <v>82448.76623670528</v>
       </c>
       <c r="D25" t="n">
-        <v>2152.340750492647</v>
+        <v>2152.340750492648</v>
       </c>
       <c r="E25" t="n">
-        <v>734242.9834594065</v>
+        <v>734242.9834594068</v>
       </c>
       <c r="F25" t="n">
         <v>616795.1510601717</v>
@@ -6455,13 +6455,13 @@
         <v>1405096.059073472</v>
       </c>
       <c r="K25" t="n">
-        <v>1633273.741364331</v>
+        <v>1633273.74136433</v>
       </c>
       <c r="L25" t="n">
         <v>2120048.97943932</v>
       </c>
       <c r="M25" t="n">
-        <v>2954704.294548088</v>
+        <v>2954704.294548087</v>
       </c>
       <c r="N25" t="n">
         <v>3145991.714963238</v>
@@ -6473,7 +6473,7 @@
         <v>3403743.784575962</v>
       </c>
       <c r="Q25" t="n">
-        <v>4381096.618849824</v>
+        <v>4381096.618849823</v>
       </c>
       <c r="R25" t="n">
         <v>4492475.975957231</v>
@@ -6482,7 +6482,7 @@
         <v>4219299.110192204</v>
       </c>
       <c r="T25" t="n">
-        <v>5191265.493906791</v>
+        <v>5191265.493906792</v>
       </c>
       <c r="U25" t="n">
         <v>5731938.204054874</v>
@@ -6517,10 +6517,10 @@
         <v>22071707.94471994</v>
       </c>
       <c r="I26" t="n">
-        <v>24715240.73297127</v>
+        <v>24715240.73297128</v>
       </c>
       <c r="J26" t="n">
-        <v>24699811.96144654</v>
+        <v>24699811.96144655</v>
       </c>
       <c r="K26" t="n">
         <v>30463695.97709324</v>
@@ -6532,7 +6532,7 @@
         <v>40510581.81579984</v>
       </c>
       <c r="N26" t="n">
-        <v>53811679.23885252</v>
+        <v>53811679.23885253</v>
       </c>
       <c r="O26" t="n">
         <v>60410898.2754401</v>
@@ -6541,7 +6541,7 @@
         <v>64281136.96495478</v>
       </c>
       <c r="Q26" t="n">
-        <v>65402435.49359562</v>
+        <v>65402435.49359561</v>
       </c>
       <c r="R26" t="n">
         <v>72129999.04375523</v>
@@ -6580,7 +6580,7 @@
         <v>2865781.03933359</v>
       </c>
       <c r="F27" t="n">
-        <v>4371989.991582193</v>
+        <v>4371989.991582194</v>
       </c>
       <c r="G27" t="n">
         <v>3373635.347081213</v>
@@ -6592,7 +6592,7 @@
         <v>5824020.602834808</v>
       </c>
       <c r="J27" t="n">
-        <v>6942732.378415408</v>
+        <v>6942732.378415409</v>
       </c>
       <c r="K27" t="n">
         <v>10139710.5456557</v>
@@ -6601,7 +6601,7 @@
         <v>12505009.25133824</v>
       </c>
       <c r="M27" t="n">
-        <v>16789077.20259919</v>
+        <v>16789077.2025992</v>
       </c>
       <c r="N27" t="n">
         <v>17990194.80226567</v>
@@ -6639,13 +6639,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>8521010.897859793</v>
+        <v>8521010.897859791</v>
       </c>
       <c r="D28" t="n">
         <v>9436961.455353202</v>
       </c>
       <c r="E28" t="n">
-        <v>11589200.72103622</v>
+        <v>11589200.72103623</v>
       </c>
       <c r="F28" t="n">
         <v>31393465.71428159</v>
@@ -6666,7 +6666,7 @@
         <v>48327012.77531453</v>
       </c>
       <c r="L28" t="n">
-        <v>57853015.47108923</v>
+        <v>57853015.47108924</v>
       </c>
       <c r="M28" t="n">
         <v>73954957.18663429</v>
@@ -6684,13 +6684,13 @@
         <v>160887305.2763616</v>
       </c>
       <c r="R28" t="n">
-        <v>187205322.2024101</v>
+        <v>187205322.20241</v>
       </c>
       <c r="S28" t="n">
         <v>216513132.4970056</v>
       </c>
       <c r="T28" t="n">
-        <v>239056694.4646816</v>
+        <v>239056694.4646817</v>
       </c>
       <c r="U28" t="n">
         <v>273120010.6472656</v>
@@ -6707,7 +6707,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4996424.431547381</v>
+        <v>4996424.43154738</v>
       </c>
       <c r="D29" t="n">
         <v>5643254.983315162</v>
@@ -6716,10 +6716,10 @@
         <v>6483459.571190402</v>
       </c>
       <c r="F29" t="n">
-        <v>9219912.749393359</v>
+        <v>9219912.749393361</v>
       </c>
       <c r="G29" t="n">
-        <v>13750001.19415262</v>
+        <v>13750001.19415261</v>
       </c>
       <c r="H29" t="n">
         <v>15782462.66789335</v>
@@ -6731,13 +6731,13 @@
         <v>17676700.12152331</v>
       </c>
       <c r="K29" t="n">
-        <v>19002431.57703422</v>
+        <v>19002431.57703421</v>
       </c>
       <c r="L29" t="n">
         <v>21937758.87188637</v>
       </c>
       <c r="M29" t="n">
-        <v>26264695.29463979</v>
+        <v>26264695.29463978</v>
       </c>
       <c r="N29" t="n">
         <v>31701750.90551578</v>
@@ -6755,13 +6755,13 @@
         <v>30375092.15153418</v>
       </c>
       <c r="S29" t="n">
-        <v>32642377.04896894</v>
+        <v>32642377.04896895</v>
       </c>
       <c r="T29" t="n">
         <v>33630182.67485842</v>
       </c>
       <c r="U29" t="n">
-        <v>35614809.86531081</v>
+        <v>35614809.8653108</v>
       </c>
       <c r="V29" t="n">
         <v>39407216.74643464</v>
@@ -6778,7 +6778,7 @@
         <v>6920473.770595578</v>
       </c>
       <c r="D30" t="n">
-        <v>9421366.8977383</v>
+        <v>9421366.897738302</v>
       </c>
       <c r="E30" t="n">
         <v>13507582.89761087</v>
@@ -6790,10 +6790,10 @@
         <v>31874686.32127539</v>
       </c>
       <c r="H30" t="n">
-        <v>33944398.98934836</v>
+        <v>33944398.98934835</v>
       </c>
       <c r="I30" t="n">
-        <v>45155900.91669762</v>
+        <v>45155900.91669761</v>
       </c>
       <c r="J30" t="n">
         <v>61365596.15717313</v>
@@ -6858,7 +6858,7 @@
         <v>615729.3704376771</v>
       </c>
       <c r="H31" t="n">
-        <v>1015879.614074217</v>
+        <v>1015879.614074218</v>
       </c>
       <c r="I31" t="n">
         <v>1258304.274480057</v>
@@ -6876,7 +6876,7 @@
         <v>4229245.083239092</v>
       </c>
       <c r="N31" t="n">
-        <v>5593773.03960159</v>
+        <v>5593773.039601591</v>
       </c>
       <c r="O31" t="n">
         <v>6776500.2344305</v>
@@ -6891,7 +6891,7 @@
         <v>4941518.478916939</v>
       </c>
       <c r="S31" t="n">
-        <v>6332675.532390718</v>
+        <v>6332675.532390717</v>
       </c>
       <c r="T31" t="n">
         <v>5475154.077773004</v>
@@ -6900,7 +6900,7 @@
         <v>5203399.45738857</v>
       </c>
       <c r="V31" t="n">
-        <v>5122044.860640233</v>
+        <v>5122044.860640234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>